<commit_message>
Fix hyphen/em-dash mismatch in dismissal basis mapping
87 cases coded as 'N/A - Plaintiff Survived' (plain hyphen) were falling
through the DISMISSAL_MAP and incorrectly classified as Other. Adding the
hyphen variant to the map moves them to 'N/A — Plaintiff Survived'.

After fix: Other category shrinks from 93 to 6 cases (Pre: 13→2, Post: 80→4).
N/A — Plaintiff Survived increases correspondingly. Binary logit unchanged
(OR_post=4.606, p<.001). All tables and figures regenerated.

Co-Authored-By: Caroline Ferguson <carolineferguson@uchicago.edu>
</commit_message>
<xml_diff>
--- a/muldrow_tables.xlsx
+++ b/muldrow_tables.xlsx
@@ -1570,17 +1570,17 @@
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>87 (22.5%)</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>11 (8.5%)</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>0 (0.0%)</t>
+          <t>76 (29.7%)</t>
         </is>
       </c>
     </row>
@@ -1614,17 +1614,17 @@
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>93 (24.1%)</t>
+          <t>6 (1.6%)</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>13 (10.0%)</t>
+          <t>2 (1.5%)</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>80 (31.2%)</t>
+          <t>4 (1.6%)</t>
         </is>
       </c>
     </row>
@@ -1884,19 +1884,19 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr"/>
@@ -1932,19 +1932,19 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>31.2%</t>
+          <t>1.6%</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr"/>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>22.6%</t>
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>43.2%</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr"/>
@@ -2335,27 +2335,27 @@
         </is>
       </c>
       <c r="B13" s="6" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>10.0%</t>
+          <t>1.5%</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>1.2%</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>2.3%</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr"/>
@@ -5361,12 +5361,12 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
@@ -5399,12 +5399,12 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
@@ -5437,12 +5437,12 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>29.7%</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
@@ -5475,12 +5475,12 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>11.2%</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>31.3%</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -5513,12 +5513,12 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>43.2%</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">

</xml_diff>